<commit_message>
feat: add Compras Proveedores to Master Excel
</commit_message>
<xml_diff>
--- a/public/plantilla_maestra.xlsx
+++ b/public/plantilla_maestra.xlsx
@@ -4,8 +4,9 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Clientes" sheetId="1" r:id="rId1"/>
-    <sheet name="Operaciones" sheetId="2" r:id="rId2"/>
-    <sheet name="Caja Chica" sheetId="3" r:id="rId3"/>
+    <sheet name="Cobranza_Clientes" sheetId="2" r:id="rId2"/>
+    <sheet name="Compras_Proveedores" sheetId="3" r:id="rId3"/>
+    <sheet name="Caja Chica" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -541,6 +542,69 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Proveedor</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Folio_Factura</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Fecha_Emision</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Fecha_Vencimiento</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Subtotal</v>
+      </c>
+      <c r="F1" t="str">
+        <v>IVA</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Total</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Estatus</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Bolsas y Empaques SA</v>
+      </c>
+      <c r="B2" t="str">
+        <v>F-9901</v>
+      </c>
+      <c r="C2" t="str">
+        <v>25/07/2026</v>
+      </c>
+      <c r="D2" t="str">
+        <v>25/08/2026</v>
+      </c>
+      <c r="E2">
+        <v>10000</v>
+      </c>
+      <c r="F2">
+        <v>1600</v>
+      </c>
+      <c r="G2">
+        <v>11600</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Pendiente</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
   <sheetData>
     <row r="1">

</xml_diff>